<commit_message>
fix: mock-run findings — P6/line sheets excluded from hierarchy, MEL claims for seeded records, parent-as-dependency dedup
</commit_message>
<xml_diff>
--- a/tests/fixtures/compiler-mel.xlsx
+++ b/tests/fixtures/compiler-mel.xlsx
@@ -409,7 +409,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H8"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -593,9 +593,35 @@
         <v>New</v>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" s="2" t="str">
+        <v>B14-FCU-7101</v>
+      </c>
+      <c r="B8" s="2" t="str">
+        <v>Fan coil unit</v>
+      </c>
+      <c r="C8" s="2" t="str">
+        <v>2201</v>
+      </c>
+      <c r="D8" s="2" t="str">
+        <v>B14</v>
+      </c>
+      <c r="E8" s="2" t="str">
+        <v>B14-AHU-7001</v>
+      </c>
+      <c r="F8" s="2" t="str">
+        <v>Mechanical</v>
+      </c>
+      <c r="G8" s="2" t="str">
+        <v>Screening</v>
+      </c>
+      <c r="H8" s="2" t="str">
+        <v>New</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H8"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: drag-to-teach — one drag generalizes to same-kind siblings by tag numbers
</commit_message>
<xml_diff>
--- a/tests/fixtures/compiler-mel.xlsx
+++ b/tests/fixtures/compiler-mel.xlsx
@@ -409,7 +409,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H13"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -723,9 +723,35 @@
         <v>New</v>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" s="2" t="str">
+        <v>B14-PT-7001-02</v>
+      </c>
+      <c r="B13" s="2" t="str">
+        <v>Pressure transmitter</v>
+      </c>
+      <c r="C13" s="2" t="str">
+        <v>2201</v>
+      </c>
+      <c r="D13" s="2" t="str">
+        <v>B14</v>
+      </c>
+      <c r="E13" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F13" s="2" t="str">
+        <v>Mechanical</v>
+      </c>
+      <c r="G13" s="2" t="str">
+        <v>Screening</v>
+      </c>
+      <c r="H13" s="2" t="str">
+        <v>New</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H12"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H13"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>